<commit_message>
Update payment links batch upload file
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_payment_links_v2.xlsx
+++ b/public/files/sample_batch_payment_links_v2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Invoice Number</t>
   </si>
@@ -25,7 +25,10 @@
     <t>Customer Contact</t>
   </si>
   <si>
-    <t>Amount (In Paise)</t>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Amount</t>
   </si>
   <si>
     <t>Description</t>
@@ -46,6 +49,9 @@
     <t>test@test.test</t>
   </si>
   <si>
+    <t>INR</t>
+  </si>
+  <si>
     <t>Test payment link's description</t>
   </si>
 </sst>
@@ -53,18 +59,25 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
-      <sz val="11.0"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
       <name val="Calibri"/>
     </font>
-    <font/>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="8.0"/>
       <color rgb="FF085296"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,14 +94,23 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -104,66 +126,63 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="18.57"/>
-    <col customWidth="1" min="2" max="2" width="16.71"/>
-    <col customWidth="1" min="3" max="3" width="21.0"/>
-    <col customWidth="1" min="4" max="4" width="23.14"/>
-    <col customWidth="1" min="5" max="5" width="12.29"/>
-    <col customWidth="1" min="6" max="6" width="13.43"/>
-    <col customWidth="1" min="7" max="7" width="14.57"/>
-    <col customWidth="1" min="8" max="8" width="28.86"/>
-  </cols>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4">
         <v>9.999988888E9</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4">
         <v>100.0</v>
       </c>
-      <c r="F2" t="s">
-        <v>11</v>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5"/>
+      <c r="I2" s="4">
         <v>0.0</v>
       </c>
     </row>
@@ -171,9 +190,6 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
   </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "Update payment links batch upload file"
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_payment_links_v2.xlsx
+++ b/public/files/sample_batch_payment_links_v2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>Invoice Number</t>
   </si>
@@ -25,10 +25,7 @@
     <t>Customer Contact</t>
   </si>
   <si>
-    <t>Currency</t>
-  </si>
-  <si>
-    <t>Amount</t>
+    <t>Amount (In Paise)</t>
   </si>
   <si>
     <t>Description</t>
@@ -49,9 +46,6 @@
     <t>test@test.test</t>
   </si>
   <si>
-    <t>INR</t>
-  </si>
-  <si>
     <t>Test payment link's description</t>
   </si>
 </sst>
@@ -59,25 +53,18 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+  <fonts count="3">
     <font>
-      <sz val="10.0"/>
+      <sz val="11.0"/>
       <color rgb="FF000000"/>
-      <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
       <name val="Calibri"/>
     </font>
+    <font/>
     <font>
       <u/>
-      <sz val="8.0"/>
+      <sz val="11.0"/>
       <color rgb="FF085296"/>
       <name val="Calibri"/>
-    </font>
-    <font>
-      <sz val="8.0"/>
-      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -94,23 +81,14 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="3">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -126,63 +104,66 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <outlinePr summaryBelow="0" summaryRight="0"/>
+    <pageSetUpPr/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
+  <cols>
+    <col customWidth="1" min="1" max="1" width="18.57"/>
+    <col customWidth="1" min="2" max="2" width="16.71"/>
+    <col customWidth="1" min="3" max="3" width="21.0"/>
+    <col customWidth="1" min="4" max="4" width="23.14"/>
+    <col customWidth="1" min="5" max="5" width="12.29"/>
+    <col customWidth="1" min="6" max="6" width="13.43"/>
+    <col customWidth="1" min="7" max="7" width="14.57"/>
+    <col customWidth="1" min="8" max="8" width="28.86"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="D2">
+        <v>9.999988888E9</v>
+      </c>
+      <c r="E2">
+        <v>100.0</v>
+      </c>
+      <c r="F2" t="s">
         <v>11</v>
       </c>
-      <c r="D2" s="4">
-        <v>9.999988888E9</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F2" s="4">
-        <v>100.0</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="H2" s="5"/>
-      <c r="I2" s="4">
+      <c r="H2">
         <v>0.0</v>
       </c>
     </row>
@@ -190,6 +171,9 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
   </hyperlinks>
+  <printOptions/>
+  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
+  <pageSetup orientation="landscape"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Revert "Revert "Update payment links batch upload file""
This reverts commit b00725fbe0a1c64adc03804f79b09036d1547cca.
</commit_message>
<xml_diff>
--- a/public/files/sample_batch_payment_links_v2.xlsx
+++ b/public/files/sample_batch_payment_links_v2.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>Invoice Number</t>
   </si>
@@ -25,7 +25,10 @@
     <t>Customer Contact</t>
   </si>
   <si>
-    <t>Amount (In Paise)</t>
+    <t>Currency</t>
+  </si>
+  <si>
+    <t>Amount</t>
   </si>
   <si>
     <t>Description</t>
@@ -46,6 +49,9 @@
     <t>test@test.test</t>
   </si>
   <si>
+    <t>INR</t>
+  </si>
+  <si>
     <t>Test payment link's description</t>
   </si>
 </sst>
@@ -53,18 +59,25 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+  <fonts count="4">
     <font>
-      <sz val="11.0"/>
+      <sz val="10.0"/>
       <color rgb="FF000000"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
       <name val="Calibri"/>
     </font>
-    <font/>
     <font>
       <u/>
-      <sz val="11.0"/>
+      <sz val="8.0"/>
       <color rgb="FF085296"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -81,14 +94,23 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment readingOrder="0"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+      <alignment horizontal="right" readingOrder="0" vertical="bottom"/>
+    </xf>
+    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -104,66 +126,63 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <sheetPr>
-    <pageSetUpPr/>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.0"/>
-  <cols>
-    <col customWidth="1" min="1" max="1" width="18.57"/>
-    <col customWidth="1" min="2" max="2" width="16.71"/>
-    <col customWidth="1" min="3" max="3" width="21.0"/>
-    <col customWidth="1" min="4" max="4" width="23.14"/>
-    <col customWidth="1" min="5" max="5" width="12.29"/>
-    <col customWidth="1" min="6" max="6" width="13.43"/>
-    <col customWidth="1" min="7" max="7" width="14.57"/>
-    <col customWidth="1" min="8" max="8" width="28.86"/>
-  </cols>
+  <sheetFormatPr customHeight="1" defaultColWidth="14.43" defaultRowHeight="15.75"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>8</v>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="s">
-        <v>8</v>
-      </c>
-      <c r="B2" t="s">
+      <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2">
+      <c r="C2" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" s="4">
         <v>9.999988888E9</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F2" s="4">
         <v>100.0</v>
       </c>
-      <c r="F2" t="s">
-        <v>11</v>
+      <c r="G2" s="1" t="s">
+        <v>13</v>
       </c>
-      <c r="H2">
+      <c r="H2" s="5"/>
+      <c r="I2" s="4">
         <v>0.0</v>
       </c>
     </row>
@@ -171,9 +190,6 @@
   <hyperlinks>
     <hyperlink r:id="rId1" ref="C2"/>
   </hyperlinks>
-  <printOptions/>
-  <pageMargins bottom="0.75" footer="0.0" header="0.0" left="0.7" right="0.7" top="0.75"/>
-  <pageSetup orientation="landscape"/>
   <drawing r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>